<commit_message>
:sparkles: Expand style extraction and rendering support
</commit_message>
<xml_diff>
--- a/src/tests/fixtures/sample_template.xlsx
+++ b/src/tests/fixtures/sample_template.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20,7 +20,7 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="DD/MM/YYYY HH:MM"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -44,8 +44,20 @@
       <color rgb="FFCC0000"/>
       <sz val="12"/>
     </font>
+    <font>
+      <strike val="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <vertAlign val="superscript"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <vertAlign val="subscript"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -67,8 +79,14 @@
         <fgColor rgb="FFCCFFCC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="gray125">
+        <fgColor rgb="FF000000"/>
+        <bgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -90,11 +108,24 @@
         <color rgb="FF000000"/>
       </bottom>
     </border>
+    <border diagonalUp="1" diagonalDown="1">
+      <diagonal style="thin">
+        <color rgb="FF000000"/>
+      </diagonal>
+    </border>
+    <border>
+      <start style="medium">
+        <color rgb="FF0000FF"/>
+      </start>
+      <end style="dashed">
+        <color rgb="FFFF0000"/>
+      </end>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -113,6 +144,24 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment indent="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment textRotation="45"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -478,7 +527,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -540,6 +589,64 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" s="10" t="inlineStr">
+        <is>
+          <t>Strikethrough</t>
+        </is>
+      </c>
+      <c r="B6" s="11" t="inlineStr">
+        <is>
+          <t>Super2</t>
+        </is>
+      </c>
+      <c r="C6" s="12" t="inlineStr">
+        <is>
+          <t>Sub2</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="13" t="inlineStr">
+        <is>
+          <t>Indented</t>
+        </is>
+      </c>
+      <c r="B7" s="14" t="inlineStr">
+        <is>
+          <t>Rotated</t>
+        </is>
+      </c>
+      <c r="C7" s="15" t="inlineStr">
+        <is>
+          <t>Shrink</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="16" t="inlineStr">
+        <is>
+          <t>RTL</t>
+        </is>
+      </c>
+      <c r="B8" s="17" t="inlineStr">
+        <is>
+          <t>Diagonal</t>
+        </is>
+      </c>
+      <c r="C8" s="18" t="inlineStr">
+        <is>
+          <t>Start/End</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="19" t="inlineStr">
+        <is>
+          <t>Pattern Fill</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:C2"/>

</xml_diff>

<commit_message>
:truck: Organize mindoff_dataport into extract/compile/render subpackages
</commit_message>
<xml_diff>
--- a/src/tests/fixtures/sample_template.xlsx
+++ b/src/tests/fixtures/sample_template.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
:zap: Speed up XLSX repeat streaming exports
</commit_message>
<xml_diff>
--- a/src/tests/fixtures/sample_template.xlsx
+++ b/src/tests/fixtures/sample_template.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
Revert "🚚 Organize mindoff_dataport into extract, compile, and render subpackages"
</commit_message>
<xml_diff>
--- a/src/tests/fixtures/sample_template.xlsx
+++ b/src/tests/fixtures/sample_template.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
:sparkles: Add repeat dataframe header support for PDF
</commit_message>
<xml_diff>
--- a/src/tests/fixtures/sample_template.xlsx
+++ b/src/tests/fixtures/sample_template.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
:test_tube: Expand repeat dataframe header test coverage
</commit_message>
<xml_diff>
--- a/src/tests/fixtures/sample_template.xlsx
+++ b/src/tests/fixtures/sample_template.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
Add fidelity export tests and benchmark comparison reporting
</commit_message>
<xml_diff>
--- a/src/tests/fixtures/sample_template.xlsx
+++ b/src/tests/fixtures/sample_template.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
:test_tube: Raise renderer and contract coverage with lean branch tests
</commit_message>
<xml_diff>
--- a/src/tests/fixtures/sample_template.xlsx
+++ b/src/tests/fixtures/sample_template.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
🧪 Increase renderer and contract test coverage with lean branch tests (#13)
</commit_message>
<xml_diff>
--- a/src/tests/fixtures/sample_template.xlsx
+++ b/src/tests/fixtures/sample_template.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
:recycle: Align test_bundle with Sonar naming and float-assert conventions
</commit_message>
<xml_diff>
--- a/src/tests/fixtures/sample_template.xlsx
+++ b/src/tests/fixtures/sample_template.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
:chart_with_upwards_trend: Update benchmark results
</commit_message>
<xml_diff>
--- a/src/tests/fixtures/sample_template.xlsx
+++ b/src/tests/fixtures/sample_template.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>